<commit_message>
Direct KZ: three campaigns (workshop search, workshop RSYa, main site search) with per-group ads, 8 sitelinks, 6 callouts, cross-minus check, placement in UTM; settings with budget, RSYa protection and launch checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KL6o371qpbTr1MgjKJCrM5
</commit_message>
<xml_diff>
--- a/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
+++ b/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Настройки" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Бюджет" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Защита РСЯ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Контроль запуска" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,10 +32,15 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000000FF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color theme="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,9 +68,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -429,22 +451,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,196 +476,700 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Места показа</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Места показа</t>
+          <t>Регион</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Регион</t>
+          <t>Даты</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Даты</t>
+          <t>Расписание (время Астаны, UTC+5)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Расписание (время Астаны, UTC+5)</t>
+          <t>Стратегия</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Стратегия</t>
+          <t>Дневной бюджет, ₽</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Недельный бюджет, ₽ (предложение)</t>
+          <t>Ставка на фразы, ₽</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Ставки</t>
+          <t>Автотаргетинг</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Автотаргетинг</t>
+          <t>Картинки</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Картинки</t>
+          <t>Посадочная</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Счётчик Метрики</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Прочее</t>
+          <t>Общее для всех</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KZ_Воркшоп_12_ноября</t>
+          <t>KZ_Воркшоп_Поиск</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Единая перфоманс-кампания</t>
+          <t>Только поиск: сети, Карты, товарная галерея — выключить</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Поиск + Рекламная сеть (решение владельца 24.10)</t>
+          <t>Казахстан</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Казахстан</t>
+          <t>С запуска до 12 ноября, 19:00 по Астане</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>С запуска до 12 ноября 19:00 по Астане</t>
+          <t>Ежедневно 8:00–23:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Ежедневно 8:00–23:00</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Максимум кликов с ручными ставками, недельный бюджет</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>≈7 000</t>
-        </is>
+          <t>Максимум кликов с ручными ставками, дневной бюджет, режим «Распределённый»</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>30</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Фразы — 30 ₽, автотаргетинг — 0,3 ₽ (как в WinWinBot KZ); в сетях — по прогнозу Коммандера</t>
+          <t>«Целевые» и «Узкие», бренды — «Без упоминания брендов», ставка 0,3 ₽</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Только «Целевые» и «Узкие», бренды — «Без упоминания брендов»</t>
+          <t>Не нужны</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Добавить 2 картинки: 1080×607 и 1080×1080 (присланы в чат, на сайт не выкладываются)</t>
+          <t>/ru/webinar</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>113476399 (цели почти не набираются — Метрика только после согласия на cookie)</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Название кампании задать вручную (из файла не берётся). «Автоматически применять рекомендации» и «Персонализация» — выключить, «Мониторинг сайта» — включить, автопометка yclid — включить.</t>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>KZ_Услуги_Поиск</t>
+          <t>KZ_Воркшоп_РСЯ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Единая перфоманс-кампания</t>
+          <t>Только Рекламная сеть: поиск выключить. Внешние сети — исключить на старте</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Только поиск (сети, Карты, галереи — выключить)</t>
+          <t>Казахстан</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>С запуска до 12 ноября, 19:00 по Астане</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ежедневно 8:00–23:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Максимум кликов с ручными ставками, дневной бюджет, режим «Распределённый»</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Только «Целевые», бренды — «Без упоминания брендов», ставка 0,3 ₽</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>12 файлов KZ_A/B/C_* (идеи A, B, C × 1:1, 16:9, 3:4, 4:3) в каждую группу</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>/ru/webinar</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KZ_Сайт_Поиск</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Только поиск: сети, Карты, товарная галерея — выключить</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Казахстан</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>С запуска, без даты окончания</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Будни 9:00–20:00</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Максимум кликов с ручными ставками, недельный бюджет</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>2 000–3 000</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Фразы — 30 ₽, автотаргетинг — 0,3 ₽</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Только «Целевые» и «Узкие», бренды — «Без упоминания брендов»</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Не нужны (только поиск)</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>113476399</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Название кампании задать вручную. Рекомендации и персонализация — выключить, мониторинг сайта и автопометка yclid — включить.</t>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Максимум кликов с ручными ставками, дневной бюджет, режим «Распределённый»</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>«Целевые» и «Узкие», бренды — «Без упоминания брендов», ставка 0,3 ₽</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Не нужны</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>/ru (главная)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Кампания</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Дневной бюджет, ₽</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>В неделю, ₽</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Дней</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Всего, ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Дата запуска (меняйте)</t>
+        </is>
+      </c>
+      <c r="B2" s="4">
+        <f>DATE(2026,10,27)</f>
+        <v/>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KZ_Воркшоп_Поиск</t>
+        </is>
+      </c>
+      <c r="B3" s="5">
+        <f>Настройки!G2</f>
+        <v/>
+      </c>
+      <c r="C3" s="5">
+        <f>B3*7</f>
+        <v/>
+      </c>
+      <c r="D3" s="2">
+        <f>DATE(2026,11,12)-$B$2+1</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>B3*D3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KZ_Воркшоп_РСЯ</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>Настройки!G3</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>B4*7</f>
+        <v/>
+      </c>
+      <c r="D4" s="2">
+        <f>DATE(2026,11,12)-$B$2+1</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>B4*D4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KZ_Сайт_Поиск</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>Настройки!G4</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>B5*7</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>DATE(2026,11,30)-$B$2+1</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>B5*D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>SUM(B3:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>SUM(C3:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="5">
+        <f>SUM(E3:E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Бюджеты — предложение, решает владелец (меняются на листе «Настройки», колонка G). Воркшоп считаем до 12 ноября, сайт — до 30 ноября. Директ может списать за день до 20% больше дневного бюджета, но не больше 7 дневных бюджетов за неделю.</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Правило</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Что сделать</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Отдельные кампании</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Поиск и РСЯ — разные кампании. Иначе сети съедают бюджет поиска и не видно, где какая цена клика.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Ручные ставки</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>«Максимум кликов с ручными ставками». Автостратегию «Максимум кликов» не ставить: в WinWinBot она в первые сутки скупила дешёвые клики автотаргетинга по мусорным запросам. Оплату за конверсии не включаем: цели Метрики почти не набираются (Метрика работает только после согласия на cookie).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Распределённый бюджет</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Режим дневного бюджета «Распределённый»: деньги не уходят в первые утренние часы.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Низкая ставка на старте</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>РСЯ — 12 ₽ за клик. Если за 2 дня мало показов, поднимать по 2–3 ₽ за раз, не больше 20 ₽ без решения владельца.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Только узкие фразы</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>В файлах фразы из 2–4 слов про бизнес и продажи, однословных нет. Минус-слова отсекают детей, учёбу, работу, игры, картинки, «вход/кабинет».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Автотаргетинг</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>В ЕПК не выключается. В РСЯ оставить только «Целевые», без брендов, ставка 0,3 ₽ — фактически не работает. Строки ---autotargeting не останавливать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Гео</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Только Казахстан, «Расширенный географический таргетинг» выключен — без показов в России.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>«Младше 18 лет» — −100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Время</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Без ночных показов: 8:00–23:00 по Астане.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Внешние сети</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Исключить на старте, включать только если РСЯ не открутит бюджет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Площадки</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Каждые 2–3 дня: Мастер отчётов → срез «Площадка» за всё время. В «Запрещённые площадки» (до 1000) — площадки с 15+ кликами без единой записи и мобильные игры. Ориентир: CTR в РСЯ выше 3% почти всегда случайные клики в приложениях.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Площадка — в CRM</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>В каждой ссылке utm_content={ad_id}_{source}: площадка видна в поле «Источник» сделки amoCRM. Площадки, с которых приходят записи, не трогаем.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Картинки</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Все 4 формата каждой из 3 идей — Директ сам подберёт размер. Через 5–7 дней худшую идею по CTR и записям отключить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Мониторинг сайта</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Включить: если сайт недоступен, Директ сам остановит показы.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Когда</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Что проверить</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>До запуска</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Проверить в каждой кампании: место показа, регион и выключенный расширенный геотаргетинг, расписание, дневной бюджет, ставки, автотаргетинг, корректировку по возрасту, картинки в группах РСЯ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>День 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Модерация пройдена, показы идут. Цена клика на поиске и в РСЯ, списание не выше дневного бюджета.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>День 2–3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Поисковые запросы → минус-слова. Площадки РСЯ → запрет. Записи на воркшоп с utm_source=yandex в amoCRM (отчёт «Проверка воронки»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>День 7</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Стоимость записи и заявки по каждой из 3 кампаний (расход Директа / сделки amoCRM с её utm_campaign). Бюджет — в кампанию с самой дешёвой записью.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>11 ноября</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Последний день записи: проверить, что бюджет воркшопа не упирается в дневной лимит.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>12 ноября, 19:00</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Кампании воркшопа останавливаются по дате окончания. Проверить, что показы прекратились.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Analytics without the cookie click on both sites (owner's decision): GA4 and Metrica load unless declined, ads pixels after consent; Direct leads reported to Metrica server-side by yclid; Metrica goals and KZ segments in the Commander settings; privacy texts updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KL6o371qpbTr1MgjKJCrM5
</commit_message>
<xml_diff>
--- a/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
+++ b/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Настройки" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Бюджет" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Защита РСЯ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Контроль запуска" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Метрика" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Защита РСЯ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Контроль запуска" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -465,7 +466,8 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -526,6 +528,11 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Цели Метрики</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Общее для всех</t>
         </is>
       </c>
@@ -584,7 +591,12 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
+          <t>Ключевая: «Воркшоп: запись (с сервера, все записи)» 674139007. Дополнительно: «Воркшоп: запись» 674138851. Ценность не задавать.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить (без неё не работают записи «с сервера»). Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
         </is>
       </c>
     </row>
@@ -642,7 +654,12 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
+          <t>Ключевая: «Воркшоп: запись (с сервера, все записи)» 674139007. Дополнительно: «Воркшоп: запись» 674138851. Ценность не задавать.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить (без неё не работают записи «с сервера»). Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
         </is>
       </c>
     </row>
@@ -700,7 +717,12 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить. Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
+          <t>Ключевая: «Заявка (с сервера, все заявки)» 674139009. Дополнительно: «Заявка» 670096899, «Запись в Cal.com (бронь состоялась)» 670499309, «Квиз: получил результат» 670147210.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Название кампании — вручную (из файла не берётся). «Расширенный географический таргетинг» — выключить. «Автоматически применять рекомендации» и «Персонализация» — выключить. «Мониторинг сайта» и автопометку yclid — включить (без неё не работают записи «с сервера»). Корректировка «младше 18 лет» — −100%. Счётчик Метрики 113476399.</t>
         </is>
       </c>
     </row>
@@ -884,6 +906,144 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Что</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Как настроено</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Счётчик</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>113476399 «Praxen AI» (praxenai.ge). С 24 октября Метрика и Google Analytics грузятся сразу, без нажатия кнопки cookie (решение владельца); до 24 октября данных мало — Метрика ждала согласия.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Запись «с сервера»</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Если посетитель пришёл из Директа (метка yclid в ссылке) и записался, сервер сайта сам передаёт запись в Метрику: цели «Воркшоп: запись (с сервера, все записи)» 674139007 и «Заявка (с сервера, все заявки)» 674139009. Так Директ видит все записи, даже если Метрику заблокировал браузер. Работает после того, как в Cloudflare добавлен секрет YM_OFFLINE_TOKEN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Цели воркшопа</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>«Воркшоп: открыл страницу» 674138829 · «Воркшоп: нажал «Занять место»» 674138830 · «Воркшоп: запись» 674138851 (браузер) · «Воркшоп: запись (с сервера, все записи)» 674139007.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Цели сайта</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>«Заявка» 670096899 · «Заявка (с сервера, все заявки)» 674139009 · «Контакт» 670097102 · «Запись в Cal.com (бронь состоялась)» 670499309 · «Квиз: получил результат» 670147210 · «Калькулятор» 670140464.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Сегменты</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>«Реклама KZ: все кампании», «Реклама KZ: Воркшоп Поиск», «Реклама KZ: Воркшоп РСЯ», «Реклама KZ: Сайт Поиск», «Казахстан: весь трафик» — выбрать сверху любого отчёта («Сегменты» → «Сохранённые»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Отчёты</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>«Источники → Директ, сводка» — расход, клики, цели по кампаниям (появится после связки с Директом). «Директ, площадки» — какие площадки РСЯ дают визиты и записи. «Метки UTM» с сегментом «Реклама KZ». «Конверсии» — цели выше. Вебвизор — записи визитов из рекламы.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Связка с Директом</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>В каждой кампании указать счётчик 113476399 и цели из листа «Настройки». Если Директ на другом логине Яндекса, чем Метрика, — в Метрике «Настройки → Доступ» дать этому логину гостевой доступ, иначе расходы в Метрику не придут.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Ретаргетинг (по желанию)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Через 5–7 дней в кампанию «Воркшоп_РСЯ» можно добавить группу с условием «Воркшоп: открыл страницу» и без «Воркшоп: запись» за 14 дней — вернуть тех, кто смотрел и не записался.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Стратегия позже</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Сейчас — клики с ручными ставками. Когда будет 10+ записей «с сервера» в неделю, можно перейти на «Оплату за конверсии» по цели 674139007 — только по решению владельца.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1076,7 +1236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Metrica funnels: workshop steps send their own goal ids (workshop_cta/form/lead), checkout and purchase goals; autogoals removed; goal ids updated in the Commander settings and docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KL6o371qpbTr1MgjKJCrM5
</commit_message>
<xml_diff>
--- a/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
+++ b/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Воркшоп: запись (с сервера, все записи)» 674139007. Дополнительно: «Воркшоп: запись» 674138851. Ценность не задавать.</t>
+          <t>Ключевая: «Воркшоп 4 · записался — все, с сервера» 674139007. Дополнительно: «Воркшоп 4 · записался» 674143270. Ценность не задавать.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Воркшоп: запись (с сервера, все записи)» 674139007. Дополнительно: «Воркшоп: запись» 674138851. Ценность не задавать.</t>
+          <t>Ключевая: «Воркшоп 4 · записался — все, с сервера» 674139007. Дополнительно: «Воркшоп 4 · записался» 674143270. Ценность не задавать.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Заявка (с сервера, все заявки)» 674139009. Дополнительно: «Заявка» 670096899, «Запись в Cal.com (бронь состоялась)» 670499309, «Квиз: получил результат» 670147210.</t>
+          <t>Ключевая: «Услуги 2 · заявка — все, с сервера» 674139009. Дополнительно: «Услуги 2 · заявка» 670096899, «Услуги 3 · записался на аудит» 670499309, «Сайт · квиз: получил результат» 670147210.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -933,101 +933,113 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>113476399 «Praxen AI» (praxenai.ge). С 24 октября Метрика и Google Analytics грузятся сразу, без нажатия кнопки cookie (решение владельца); до 24 октября данных мало — Метрика ждала согласия.</t>
+          <t>113476399 «Praxen AI» (praxenai.ge). С 24 октября Метрика и Google Analytics грузятся сразу, без нажатия кнопки cookie (решение владельца). Автоцели выключены и удалены — только свои цели ниже.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Запись «с сервера»</t>
+          <t>Воронка воркшопа</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Если посетитель пришёл из Директа (метка yclid в ссылке) и записался, сервер сайта сам передаёт запись в Метрику: цели «Воркшоп: запись (с сервера, все записи)» 674139007 и «Заявка (с сервера, все заявки)» 674139009. Так Директ видит все записи, даже если Метрику заблокировал браузер. Работает после того, как в Cloudflare добавлен секрет YM_OFFLINE_TOKEN.</t>
+          <t>Воркшоп 1 · открыл страницу 674138829 → 2 · нажал «Занять место» 674143265 → 3 · начал заполнять форму 674143266 → 4 · записался 674143270 (и «— все, с сервера» 674139007) → 5 · открыл тарифы 674143271 → 6 · начал оплату 674143274 → 7 · оплатил 674143277. Конверсия по шагам за один визит — составная цель «Воронка воркшопа» 674143279.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Цели воркшопа</t>
+          <t>Воронка услуг</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>«Воркшоп: открыл страницу» 674138829 · «Воркшоп: нажал «Занять место»» 674138830 · «Воркшоп: запись» 674138851 (браузер) · «Воркшоп: запись (с сервера, все записи)» 674139007.</t>
+          <t>Услуги 1 · начал заполнять форму 670140446 → 2 · заявка 670096899 (и «— все, с сервера» 674139009) → 3 · записался на аудит 670499309. Составная цель «Воронка услуг» 674143286. Записи на воркшоп в эту воронку не попадают.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Цели сайта</t>
+          <t>Запись «с сервера»</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>«Заявка» 670096899 · «Заявка (с сервера, все заявки)» 674139009 · «Контакт» 670097102 · «Запись в Cal.com (бронь состоялась)» 670499309 · «Квиз: получил результат» 670147210 · «Калькулятор» 670140464.</t>
+          <t>Если посетитель пришёл из Директа (метка yclid в ссылке) и записался, сервер сайта сам передаёт запись в Метрику (цели «… — все, с сервера»). Так Директ видит все записи, даже если Метрику заблокировал браузер. Секрет YM_OFFLINE_TOKEN в Cloudflare добавлен, проверено 24 октября.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Сегменты</t>
+          <t>Прочие цели</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>«Реклама KZ: все кампании», «Реклама KZ: Воркшоп Поиск», «Реклама KZ: Воркшоп РСЯ», «Реклама KZ: Сайт Поиск», «Казахстан: весь трафик» — выбрать сверху любого отчёта («Сегменты» → «Сохранённые»).</t>
+          <t>Контакт · любой / WhatsApp / Telegram / звонок / открыл запись в Cal.com; Сайт · калькулятор, клик «Бесплатный аудит», квиз: начал, квиз: получил результат.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Отчёты</t>
+          <t>Сегменты</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>«Источники → Директ, сводка» — расход, клики, цели по кампаниям (появится после связки с Директом). «Директ, площадки» — какие площадки РСЯ дают визиты и записи. «Метки UTM» с сегментом «Реклама KZ». «Конверсии» — цели выше. Вебвизор — записи визитов из рекламы.</t>
+          <t>«Реклама KZ: все кампании», «Реклама KZ: Воркшоп Поиск», «Реклама KZ: Воркшоп РСЯ», «Реклама KZ: Сайт Поиск», «Казахстан: весь трафик» — выбрать сверху любого отчёта («Сегменты» → «Сохранённые»).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Связка с Директом</t>
+          <t>Отчёты</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>В каждой кампании указать счётчик 113476399 и цели из листа «Настройки». Если Директ на другом логине Яндекса, чем Метрика, — в Метрике «Настройки → Доступ» дать этому логину гостевой доступ, иначе расходы в Метрику не придут.</t>
+          <t>«Обзор» — блоки «Все источники, кроме рекламы» и «Контекстная реклама» с целями воронок. «Источники → Директ, сводка» — расход, клики, цели по кампаниям. «Директ, площадки» — какие площадки РСЯ дают визиты и записи. «Конверсии» — шаги воронок. Вебвизор — записи визитов из рекламы.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Ретаргетинг (по желанию)</t>
+          <t>Связка с Директом</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Через 5–7 дней в кампанию «Воркшоп_РСЯ» можно добавить группу с условием «Воркшоп: открыл страницу» и без «Воркшоп: запись» за 14 дней — вернуть тех, кто смотрел и не записался.</t>
+          <t>В каждой кампании указать счётчик 113476399 и цели из листа «Настройки». Если Директ на другом логине Яндекса, чем Метрика, — в Метрике «Настройки → Доступ» дать этому логину гостевой доступ, иначе расходы в Метрику не придут.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Ретаргетинг (по желанию)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Через 5–7 дней в кампанию «Воркшоп_РСЯ» можно добавить группу с условием «Воркшоп 1 · открыл страницу» и без «Воркшоп 4 · записался — все, с сервера» за 14 дней.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Стратегия позже</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Сейчас — клики с ручными ставками. Когда будет 10+ записей «с сервера» в неделю, можно перейти на «Оплату за конверсии» по цели 674139007 — только по решению владельца.</t>
         </is>

</xml_diff>

<commit_message>
Metrica: service enquiries reach their own goals (training, implementation, development, maintenance) from the tariff the visitor came from; purchase goal carries revenue; goal names and ids updated in the Commander settings and docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KL6o371qpbTr1MgjKJCrM5
</commit_message>
<xml_diff>
--- a/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
+++ b/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Воркшоп 4 · записался — все, с сервера» 674139007. Дополнительно: «Воркшоп 4 · записался» 674143270. Ценность не задавать.</t>
+          <t>Ключевая: «Воркшоп · зарегистрировался» 674143270. Ценность не задавать.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Воркшоп 4 · записался — все, с сервера» 674139007. Дополнительно: «Воркшоп 4 · записался» 674143270. Ценность не задавать.</t>
+          <t>Ключевая: «Воркшоп · зарегистрировался» 674143270. Ценность не задавать.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Ключевая: «Услуги 2 · заявка — все, с сервера» 674139009. Дополнительно: «Услуги 2 · заявка» 670096899, «Услуги 3 · записался на аудит» 670499309, «Сайт · квиз: получил результат» 670147210.</t>
+          <t>Ключевая: «Сайт · заявка (любая услуга)» 670096899. Дополнительно: «Бесплатный аудит · забронировал время» 670499309 и заявки по услугам: «Обучение команды» 674307503, «Внедрение инструментов» 674307641, «Разработка решения» 674307642, «Дополнительное ведение» 674307643.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -933,50 +933,50 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>113476399 «Praxen AI» (praxenai.ge). С 24 октября Метрика и Google Analytics грузятся сразу, без нажатия кнопки cookie (решение владельца). Автоцели выключены и удалены — только свои цели ниже.</t>
+          <t>113476399 «Praxen AI» (praxenai.ge). С 24 октября Метрика и Google Analytics грузятся сразу, без нажатия кнопки cookie (решение владельца). Автоцели выключены и удалены.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Воронка воркшопа</t>
+          <t>Воркшоп</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Воркшоп 1 · открыл страницу 674138829 → 2 · нажал «Занять место» 674143265 → 3 · начал заполнять форму 674143266 → 4 · записался 674143270 (и «— все, с сервера» 674139007) → 5 · открыл тарифы 674143271 → 6 · начал оплату 674143274 → 7 · оплатил 674143277. Конверсия по шагам за один визит — составная цель «Воронка воркшопа» 674143279.</t>
+          <t>Воркшоп · открыл страницу 674138829 → нажал «Занять место» 674143265 → начал заполнять форму 674143266 → зарегистрировался 674143270 → открыл тарифы 674143271 → выбрал тариф или бронь 674143274 → подтверждённая оплата 674143277 (с суммой — для выручки).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Воронка услуг</t>
+          <t>Сайт</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Услуги 1 · начал заполнять форму 670140446 → 2 · заявка 670096899 (и «— все, с сервера» 674139009) → 3 · записался на аудит 670499309. Составная цель «Воронка услуг» 674143286. Записи на воркшоп в эту воронку не попадают.</t>
+          <t>Сайт · открыл страницу (не воркшоп) 674309236 → начал заполнять форму 670140446 → заявка (любая услуга) 670096899 → Бесплатный аудит · забронировал время 670499309. Записи на воркшоп сюда не попадают.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Запись «с сервера»</t>
+          <t>Заявки по услугам</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Если посетитель пришёл из Директа (метка yclid в ссылке) и записался, сервер сайта сам передаёт запись в Метрику (цели «… — все, с сервера»). Так Директ видит все записи, даже если Метрику заблокировал браузер. Секрет YM_OFFLINE_TOKEN в Cloudflare добавлен, проверено 24 октября.</t>
+          <t>Обучение команды · заявка 674307503, Внедрение инструментов · заявка 674307641, Разработка решения · заявка 674307642, Дополнительное ведение · заявка 674307643 — по кнопке тарифа, с которой пришёл человек, или по странице «Обучение». Заявка без выбранного тарифа считается только в «Сайт · заявка».</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Прочие цели</t>
+          <t>Прочие</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>«Обзор» — блоки «Все источники, кроме рекламы» и «Контекстная реклама» с целями воронок. «Источники → Директ, сводка» — расход, клики, цели по кампаниям. «Директ, площадки» — какие площадки РСЯ дают визиты и записи. «Конверсии» — шаги воронок. Вебвизор — записи визитов из рекламы.</t>
+          <t>«Обзор» — блоки по воркшопу и сайту. «Источники → Директ, сводка» — расход, клики, цели по кампаниям. «Директ, площадки» — какие площадки РСЯ дают визиты и записи. «Конверсии» — все цели. Вебвизор — записи визитов.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Через 5–7 дней в кампанию «Воркшоп_РСЯ» можно добавить группу с условием «Воркшоп 1 · открыл страницу» и без «Воркшоп 4 · записался — все, с сервера» за 14 дней.</t>
+          <t>Через 5–7 дней в кампанию «Воркшоп_РСЯ» можно добавить группу с условием «Воркшоп · открыл страницу» и без «Воркшоп · зарегистрировался» за 14 дней.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Сейчас — клики с ручными ставками. Когда будет 10+ записей «с сервера» в неделю, можно перейти на «Оплату за конверсии» по цели 674139007 — только по решению владельца.</t>
+          <t>Сейчас — клики с ручными ставками. Когда будет 10+ регистраций из рекламы в неделю, можно перейти на «Оплату за конверсии» по цели 674143270 — только по решению владельца.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Direct KZ: two more RSYa creatives with other pains (CRM chaos, routine questions), 20 images in total; settings and instructions updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KL6o371qpbTr1MgjKJCrM5
</commit_message>
<xml_diff>
--- a/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
+++ b/docs/direct-kz/commander/Настройки_кампаний_KZ.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>12 файлов KZ_A/B/C_* (идеи A, B, C × 1:1, 16:9, 3:4, 4:3) в каждую группу</t>
+          <t>20 файлов KZ_A…E_* (5 идей — 5 болей × 1:1, 16:9, 3:4, 4:3) в каждую группу</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Все 4 формата каждой из 3 идей — Директ сам подберёт размер. Через 5–7 дней худшую идею по CTR и записям отключить.</t>
+          <t>Все 4 формата каждой из 5 идей (5 разных болей) — Директ сам подберёт размер. Через 5–7 дней две худшие идеи по CTR и записям отключить.</t>
         </is>
       </c>
     </row>

</xml_diff>